<commit_message>
fix(fixtures): replace third-party personal data with fictional values
The challenge_sparse_rows.xlsx fixture and the checks and docs built from it
reproduced a row from a partner's private test workbook, naming a real third
party. That data was shared to reproduce a bug, not for publication.

Replaced everywhere with invented values that keep the same shape: blanks,
column positions and value types are unchanged, so every check still tests
exactly the same thing. The fixture was regenerated from the fixed generator,
and the regenerated golden matches the text-replaced one.

Checks: office suite 100% (112 files), check_structure_gate.py,
check_xlsx_positions.py, --check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015F4aUg2mj63Dc46HNYMtze
</commit_message>
<xml_diff>
--- a/data/test_files/challenge/challenge_sparse_rows.xlsx
+++ b/data/test_files/challenge/challenge_sparse_rows.xlsx
@@ -222,22 +222,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Adapt</t>
+          <t>ExampleCo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>adaptagency.com</t>
+          <t>example-co.example</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Kresten Finsen Wiinblad</t>
+          <t>Sam Placeholder</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -247,7 +247,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>LinkedIn outreach, 3 July 2026</t>
+          <t>Intro call, 3 July 2026</t>
         </is>
       </c>
     </row>

</xml_diff>